<commit_message>
Initial version Employee roster
</commit_message>
<xml_diff>
--- a/Workspace_FloorPlan_Template.xlsx
+++ b/Workspace_FloorPlan_Template.xlsx
@@ -28971,10 +28971,10 @@
   </sheetData>
   <conditionalFormatting sqref="H2:I401">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$G2="Yes"</formula>
+      <formula>UPPER(TRIM($G2))="YES"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>$G2&lt;&gt;"Yes"</formula>
+      <formula>UPPER(TRIM($G2))&lt;&gt;"YES"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
@@ -28985,10 +28985,10 @@
       <formula1>=F2&lt;=E2</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H401" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Meeting Room Disabled" error="Meeting Room is set to 'No' or blank. Set 'Meeting Room (Yes or No)' to 'Yes' to enter meeting room cubicles." type="custom">
-      <formula1>=$G2="Yes"</formula1>
+      <formula1>=UPPER(TRIM($G2))="YES"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I401" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Meeting Room HDMI" error="Meeting Room is set to 'No', or HDMI count exceeds Meeting Room cubicle capacity." type="custom">
-      <formula1>=AND($G2="Yes", I2&lt;=H2)</formula1>
+      <formula1>=AND(UPPER(TRIM($G2))="YES", I2&lt;=H2)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>